<commit_message>
Global Search cases: adversarial review corrections
Rule-9 wording fixes found in adversarial review:
- GS-FUZ-02: replace invented label "Abridge" with spec's actual
  "Aabridge" (requirements.md §1); title/precond/expected + coverage-matrix.
- GS-FUZ-10: soft-match symbol "~" corrected to spec's "≈" (requirements.md §7)
  in expected/design_ref/notes.
Regenerated GlobalSearch_TestRail-Import.csv/.xlsx from gen_import.py
(84 cases, 15 sections, VIU-word-free, flag-free, API cases API-placed).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/global-search/GlobalSearch_TestRail-Import.xlsx
+++ b/build/global-search/GlobalSearch_TestRail-Import.xlsx
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>A misspelled name still finds the record - 'Abrige' finds 'Abridge'</t>
+          <t>A misspelled name still finds the record - 'Abrige' finds 'Aabridge'</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2447,7 +2447,7 @@
       <c r="E36" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
-2. A record whose name contains 'Abridge' (for example 'Aabridge') exists.</t>
+2. A record whose name contains 'Aabridge' exists.</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>1. The 'Abridge' / 'Aabridge' record is found and shown, despite the typo.</t>
+          <t>1. The 'Aabridge' record is found and shown, despite the typo.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2907,7 +2907,7 @@
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>1. The matched token is highlighted.
-2. A subtle soft-match indicator is shown for fuzzy matches (spec mentions a '~' symbol or italic treatment).</t>
+2. A subtle soft-match indicator is shown for fuzzy matches (spec mentions a '≈' symbol or italic treatment).</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Global Search: add GS-FUZ-11 (P-number exact-only) + GS-PERM-05 (sparse empty entity), regen deliverables (84->86)
Adds two coverage-completeness cases and closes the two reviewer follow-up gaps
(P-number exact-only; sparse-data empty-entity). Regenerated the TestRail import
(86 rows), updated coverage-matrix, testrail-id-map, and PROJECT-STATE counts.
LOCAL ONLY - no TestRail push.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/global-search/GlobalSearch_TestRail-Import.xlsx
+++ b/build/global-search/GlobalSearch_TestRail-Import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2930,317 +2930,373 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>Fuzzy Matching</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>A Part Sale P-number requires an exact match (no fuzzy typo tolerance)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>1. The palette is open.
+2. A Part Sale 'P2-58' exists and no Part Sale 'P2-59' exists.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>1. Type the exact P-number 'P2-58' and read the result.
+2. Clear the input, type a near-miss P-number 'P2-59' (one digit off a real Part Sale), and read the results.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>1. The exact P-number 'P2-58' finds the matching Part Sale.
+2. A one-digit-off P-number does NOT return the real Part Sale as a fuzzy match - P-numbers are exact-only identifiers, no typo tolerance (it may show 'No results' if nothing else matches).</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>GS-FUZ-11</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>Ranking and Prioritization</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>An exact identifier match is pinned as a single row at the very top</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. A Work Order 'S2-15276' exists.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. Type the exact Work Order number 'S2-15276'.
 2. Look at the top of the results.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>1. The exactly-matched Work Order is pinned as a single row at the very top, above the grouped results, labeled with its entity icon.
 2. This gives the 'type the number, jump straight to it' experience.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.2 (ID match &gt; 0.95 pinned at top)</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>GS-RANK-01</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Ranking and Prioritization</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Within a group, more relevant results appear first</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. Several Work Orders match the query, some open/active (Approved, In Progress, Review) and recently updated, some old and Completed/Invoiced.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Type a query that matches many Work Orders.
 2. Read the order of the Work Order rows.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>1. Open/active and recently-updated Work Orders rank above old, closed ones.
 2. Work Orders assigned to or recently viewed by the signed-in user are boosted; closed/Invoiced Work Orders older than 90 days are pushed down.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.1 Work Orders signals (open status +0.30, recency, assigned/viewed, old-closed demoted)</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>GS-RANK-02</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Ranking and Prioritization</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>In-stock parts rank above out-of-stock parts (out-of-stock not hidden)</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. Two parts match the query - one in stock, one out of stock.</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>1. Type a query that matches both parts.
 2. Read the order of the Part rows.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>1. The in-stock part ranks above the out-of-stock part.
 2. The out-of-stock part is still shown (out-of-stock parts are not demoted below relevance and are not hidden).</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.1 Parts signals</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>GS-RANK-03</t>
         </is>
       </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Ranking and Prioritization</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>On a Customer page, that customer's assets and work orders are boosted</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>1. You are on a specific Customer's page.
 2. That customer owns some assets and work orders, and other customers have similar-matching assets/work orders.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. While on the Customer page, open the palette and type a query that matches assets/work orders belonging to several customers.
 2. Read the ranking of the asset and work-order results.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>1. Assets and Work Orders owned by the customer whose page you are on are boosted (appear higher) compared to the same search run from an unrelated page.
 2. This is a lightweight, single contextual-bias signal.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.3 Contextual bias</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>GS-RANK-04</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Ranking and Prioritization</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>On a Work Order page, parts already on that work order are pushed down</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. You are on a specific Work Order's page.
 2. That work order already has some parts on it, and other similar-matching parts exist that are not on it.</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. While on the Work Order page, open the palette and search for parts.
 2. Read the ranking of the part results.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>1. Parts already on that work order are pushed down (demoted) relative to other matching parts.
 2. Other parts in the same category as the work order's existing parts get a small boost.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.3 Contextual bias</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>GS-RANK-05</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Empty and First-Time State</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>First-time empty state shows the placeholder, helper text and three quick-create buttons</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as a user with no recent search activity.
 2. The palette is open and the input is empty.</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette without typing anything.
 2. Read the placeholder, the helper text, and the buttons.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>1. The input shows the placeholder 'Search or ask a question'.
 2. Helper text below the input reads 'Type to start searching for work orders, parts, customers and more'.
@@ -3248,57 +3304,57 @@
 4. The footer keyboard legend is visible.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 1 (First-time search)</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>GS-EMPTY-01</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Empty and First-Time State</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>The quick-create buttons in the empty state start the matching create flow</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open in the empty state showing the three quick-create buttons.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>1. Click 'New work order' and observe.
 2. Reopen the palette, click 'New customer' and observe.
 3. Reopen the palette, click 'New inventory part' and observe.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>1. 'New work order' starts the create-work-order flow.
 2. 'New customer' starts the create-customer flow.
@@ -3306,282 +3362,282 @@
 4. None of the buttons perform a destructive action.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 1 (quick-create chips)</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>GS-EMPTY-02</t>
         </is>
       </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Recent Activity Default State</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Recent activity is grouped under Today, Yesterday, Past week and Past 30 days</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as a user who has recently opened several records (across different days).
 2. The palette is open and the input is empty.</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette without typing anything.
 2. Read the group headings and the rows under them.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>1. Instead of the first-time helper text, the palette shows your recent activity.
 2. Rows are grouped under time headings: 'Today', 'Yesterday', 'Past week', 'Past 30 days'.
 3. Each row is a previously opened record (not just a previous search word).</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 2 (Recent searches grouped by interval); 8 (persist recent-entity-views 30 days)</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>GS-REC-01</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Recent Activity Default State</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Recent activity mixes different entity types using the same row template</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>1. You have recently opened records of different types (work orders, assets, customers, parts, part sales, vendors).
 2. The palette is open and empty.</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette without typing.
 2. Read the recent rows across the time groups.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>1. Recent rows include a mix of entity types (for example a Work Order, an Asset, a Customer, a Part, a Vendor).
 2. Each recent row uses the same row template as a normal result row (icon, primary line, secondary line, status/quantity cluster).
 3. Example rows: WO 'S1-644 Fisquare Farms' [Approved], Asset '2025 Freightliner M2 - Bryan Smith', Customer 'Adale Transport' with a doc chip, Part 'Rear Shock 65547' [72], Vendor 'Report Beverages'.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 2 (same row template as a result row)</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>GS-REC-02</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Recent Activity Default State</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Clicking a recent item opens that record</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open and empty, showing recent activity.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>1. Click a recent item (for example the Work Order 'S1-644 Fisquare Farms').
 2. Watch the screen.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>1. The palette closes and the clicked record opens.
 2. Opening the record refreshes its position in recent activity (it is 'touched').</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>requirements.md 10 Phase 4 (records a touch on every result click / entity-page visit)</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>GS-REC-03</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Persisting Query</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>The typed query is retained in the header search field after the palette closes</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. You have typed a query (for example 'Fibridge') that returns results.</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>1. Type 'Fibridge' so results appear.
 2. Close the palette (press Esc or click a result).
 3. Look at the header search field.</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>1. After closing, the header search field still shows the last query 'Fibridge' as plain text.
 2. A small count badge (for example '1') is shown beside the persisted query.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 5 (Persisting search); 8 (persist last query, rehydrate on reopen)</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>GS-PERS-01</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Persisting Query</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>Reopening the palette restores the last query, scope tab and result list</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>1. You have just searched (for example 'Fibridge'), selected a scope tab, and closed the palette (the query persists in the header field).</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1. Click the header search field again (or press Cmd+K).
 2. Look at the input, the scope tab, and the results.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>1. The palette reopens with the last query 'Fibridge' already in the input.
 2. The previously selected scope tab is restored.
@@ -3589,620 +3645,620 @@
 4. The query text may appear selected/highlighted in the input so it can be replaced by typing.</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 5 (Reopening restores the query, the scope tab, and the result list)</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>GS-PERS-02</t>
         </is>
       </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Persisting Query</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>The persisted query can be cleared with the clear (x) button</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open with a persisted query (for example 'Fibridge') in the input and a clear (x) button at the right of the input.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1. Click the clear (x) button at the right of the input.
 2. Look at the input and the results.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>1. The input is cleared to empty.
 2. The results clear and the palette returns to the empty / recent-activity state (placeholder 'Search or ask a question').
 3. The persisted query is removed from the header field.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 5; design-notes screenshot 9 (clearable via the x button)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>GS-PERS-03</t>
         </is>
       </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>No-Results State</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>No matches shows 'No results for &lt;query&gt;' plus the three quick-create buttons</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. You will type a query that matches nothing (for example 'S1- 56438').</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>1. Type a query with no matches (for example 'S1- 56438').
 2. Read the centered message and the buttons.</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>1. A centered message reads 'No results for \'S1- 56438\'' (the exact query is echoed in quotes).
 2. The three quick-create buttons are shown: 'New work order', 'New customer', 'New inventory part'.
 3. The footer keyboard legend is still visible.</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 4 (No results for &lt;query&gt; + quick-create chips)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>GS-NORES-01</t>
         </is>
       </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>No-Results State</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>A quick-create button in the no-results state starts the create flow</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>1. The palette is showing the no-results state with the three quick-create buttons.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>1. Click 'New work order' (or 'New customer' / 'New inventory part').
 2. Watch the screen.</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. The matching create flow starts (create work order / customer / inventory part).
 2. No destructive action occurs.</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.2 State 4</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>GS-NORES-02</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>Hovering a Work Order result shows an 'Add new line' action</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open showing at least one Work Order row (in results or in recent activity).
 2. A pointer (mouse) is available.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over a Work Order row (for example 'S1-644 Fisquare Farms').
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>1. A right-aligned 'Add new line' button appears on hover.
 2. The action is non-destructive.</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Work Order -&gt; 'Add new line', only when currently editing a WO elsewhere)</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-01</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Hovering an Asset result shows 'New work order' plus history and checklist icons</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open showing at least one Asset row.
 2. A pointer is available.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over an Asset row (for example '2025 Freightliner M2 - Fisquare Farms').
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>1. A 'New work order' button appears on hover.
 2. Two secondary icon buttons appear: a clock/history icon and a checklist/tasks icon.
 3. The actions are non-destructive.</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Asset -&gt; 'New work order' + clock (history) and Invoice icons)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-02</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Hovering a Customer result shows 'New work order' (and 'New contact')</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open showing at least one Customer row.
 2. A pointer is available.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over a Customer row (for example 'Adale Transport').
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>1. A 'New work order' button appears on hover.
 2. A 'New contact' action is available for the customer (per spec).
 3. The actions are non-destructive.</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Customer -&gt; 'New work order', 'New contact')</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-03</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Hovering a catalog part result shows 'Add part'</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open showing a catalog part-style row.
 2. You are NOT currently editing a work order.
 3. A pointer is available.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over a catalog part row (for example 'P2-58 Toboro Industries').
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>1. An 'Add part' button appears on hover.
 2. The action is non-destructive.</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Part -&gt; 'Add part' when not currently editing a WO)</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-04</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>Hovering a Vendor result shows 'Add contact'</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open showing at least one Vendor row.
 2. A pointer is available.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over a Vendor row (for example 'Report Beverages').
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>1. An 'Add contact' button appears on hover.
 2. The action is non-destructive.</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Vendor -&gt; 'Add contact')</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-05</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Hovering an inventory part while editing a work order shows 'Add to work order'</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>1. You are currently editing a work order.
 2. The palette is open showing an inventory part row (for example 'Rear Shock 65547' with a '72' quantity chip).
 3. A pointer is available.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>1. Move the pointer over an inventory part row.
 2. Look at the right side of the row.</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>1. An 'Add to work order' button appears on hover.
 2. Using it adds the part to the work order you are editing (an inline add, non-destructive).</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Part -&gt; 'Add to work order' only when currently editing a WO)</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-06</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>Hover Quick-Actions</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>Hover quick-actions never trigger a destructive operation</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open with rows across several entity types.</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>1. Hover each entity row type and review the available quick-action buttons.
 2. Note that every quick action is an add/create-style action.</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>1. No quick action deletes, voids, or otherwise destroys data.
 2. Every action offered by a quick action is also reachable from the entity's full record (hover is non-essential).</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>requirements.md 5.4 (Quick actions never trigger destructive operations; hover state non-essential)</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>GS-HOVER-07</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>In-Page Work Orders List Search</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Searching the in-page Work Orders list filters the list and shows a matching banner</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>1. You are on the Work Orders list page (not the global search palette).
 2. Work Orders exist whose text contains 'Fib'.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>1. Type 'Fib' into the in-page Work Orders list search field.
 2. Read the list and the banner above it.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>1. The Work Orders list filters to only rows matching 'Fib'.
 2. A blue banner reads 'Showing 12 work orders matching \'Fib\'' (the count reflects the number of matches).
@@ -4210,562 +4266,620 @@
 4. The list columns remain: On Site, Status, Number, Customer, Asset, Unit, VIN/Serial #, Progress, Service Advisor, Lead Technician, Clocked In, Lines, Total Price.</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>design-notes screenshot 1 (in-page Work Orders list search banner)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>GS-LIST-01</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>In-Page Work Orders List Search</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>'Clear search' restores the full in-page Work Orders list</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>1. The Work Orders list is filtered by an in-page search (banner 'Showing N work orders matching &lt;q&gt;' is visible).</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>1. Click the 'Clear search' link in the banner.
 2. Read the list and the banner.</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>1. The filter is removed and the full Work Orders list is shown again.
 2. The 'Showing N work orders matching &lt;q&gt;' banner is removed.</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>design-notes screenshot 1</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>GS-LIST-02</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Error State</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>A search failure shows the 'Search unavailable, retry' banner</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. A network/backend failure of the search request can be simulated (for example offline the network or block the search endpoint).</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>1. With the search backend unreachable, type a query.
 2. Read the message shown in the palette.
 3. Restore connectivity and use the retry affordance.</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>1. An inline banner reads 'Search unavailable, retry'.
 2. The palette degrades gracefully - it does not crash or show a blank screen.
 3. Retrying after connectivity is restored re-runs the search and shows results.</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>requirements.md 8 (tolerate offline/network failures with an inline 'Search unavailable, retry' banner)</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>GS-ERR-01</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>Permissions and Role-Based Scoping</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>A user WITH Parts access sees Parts results in the palette</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as a user whose role includes Parts access.
 2. Parts exist that match the query.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette and type a query that matches parts.
 2. Read the results (on the 'All' tab and the 'Parts' tab).</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>1. A 'Parts' group appears with matching part rows.
 2. The 'Parts' scope tab shows the part results.</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>requirements.md 9 (all result fields respect role-based-access checks)</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>GS-PERM-01</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>Permissions and Role-Based Scoping</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>A technician WITHOUT Parts access does NOT see Parts results</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as a user whose role does NOT include Parts access.
 2. Parts exist that would match the query (verified visible to a Parts-enabled user).</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette and type a query that matches parts.
 2. Read the results (on the 'All' tab and check the 'Parts' tab).</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>1. No 'Parts' group appears and no part rows are shown.
 2. The user cannot see part results they are not permitted to access, even though those parts exist.
 3. Results for entity types the user CAN access still appear normally.</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>requirements.md 9 (a technician without Parts access does not see Parts results)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>GS-PERM-02</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>Permissions and Role-Based Scoping</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>A user WITHOUT Work Orders access does NOT see Work Order results</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as a user whose role does NOT include Work Orders access.
 2. Work Orders exist that would match the query.</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette and type a query that matches Work Orders.
 2. Read the results (the 'All' tab and the 'Work Orders' tab).</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>1. No 'Work orders' group appears and no Work Order rows are shown.
 2. Results for entity types the user CAN access still appear normally.</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>requirements.md 9 (all result fields respect role-based-access checks)</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>GS-PERM-03</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>Permissions and Role-Based Scoping</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>Results are limited to the signed-in user's own tenant</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to one tenant/organization.
 2. Records with the same searchable text exist under a different tenant.</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>1. Open the palette and type a query.
 2. Read the results.</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>1. Only records belonging to your own tenant/organization are returned.
 2. No records from any other tenant are shown (tenant isolation is respected).</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>requirements.md 9 (all result fields respect existing tenant-isolation checks)</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>GS-PERM-04</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Permissions and Role-Based Scoping</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>An entity type with no accessible records shows no group (and its scope tab shows the empty state)</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in as a user who has zero accessible records of one entity type (for example the tenant has no Part Sales yet, or the user's role scopes an entity type down to no records).
+2. Other entity types do have matching records for the query.</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the palette and type a query on the 'All' tab.
+2. Read the grouped results and confirm the empty entity type has no group.
+3. Open the scope tab for the empty entity type (for example the 'Part Sales' tab).</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>1. On the 'All' tab, no group appears for the entity type that has zero accessible results (the empty group is simply not shown).
+2. Groups for the entity types that do have matches still appear normally.
+3. The empty entity type's scope tab shows its empty / no-results treatment rather than an error.</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md 9 (must work for a single-tenant dataset where any entity type is empty, e.g. no part sales yet)</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>GS-PERM-05</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>GET /api/search returns grouped results for scope=all</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint with a valid session.
 2. Test data exists so a query matches multiple entity types.</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set to the query and scope set to 'all'.
 2. Inspect the HTTP status and the response body.</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>1. The response returns HTTP 200.
 2. The body is a grouped, ranked, scored payload containing groups for the matching entity types.
 3. Each group includes the per-item metadata needed to render rows without extra fetches.</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>requirements.md 10 Phase 1 (GET /api/search; scope=all)</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>GS-API-01</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>The scope parameter restricts GET /api/search to a single entity type</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A query matches multiple entity types.</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set and scope set to 'work_orders'.
 2. Inspect the response.
 3. Repeat with scope set to each of 'customers', 'assets', 'parts', 'vendors', 'part_sales'.</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>1. Each call returns HTTP 200.
 2. Each response contains results only for the requested scope's entity type.
 3. The accepted scope values are all, work_orders, customers, assets, parts, vendors, part_sales.</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>requirements.md 10 Phase 1 (scope parameter)</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>GS-API-02</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>GET /api/search caps each group at the limit (default 5) and returns per-group totals</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A query matches more than five records of one entity type (for example twelve Work Orders).</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set and no limit parameter.
 2. Inspect the number of rows returned for the over-full group and the total field.
 3. Repeat with limit set to a smaller value (for example 3).</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>1. With no limit, each group returns at most 5 rows (the default per-group cap).
 2. Each group reports its full total count (for example total 12) even though only 5 rows are returned.
 3. Setting limit changes the per-group cap accordingly.</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>requirements.md 10 Phase 1 (limit default 5; response includes per-group totals)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>GS-API-03</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>GET /api/search matches identifier fields exactly after normalization</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A Work Order 'S2-15276' exists.</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set to 'S2-15276'.
 2. Send GET /api/search with q set to 's215276' (no dash).
@@ -4773,487 +4887,487 @@
 4. Compare the matched Work Order in each response.</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>1. All three requests return HTTP 200 and match the same Work Order 'S2-15276'.
 2. The identifier is normalized (case, diacritics, non-alphanumerics stripped) before matching.
 3. The exact-match result scores high enough to be flagged as the pinned top match (score above 0.95).</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>requirements.md 7 (identifier normalization); 6.2 (ID match pinned)</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>GS-API-04</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>GET /api/search does NOT apply fuzzy matching to identifier fields</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A Work Order 'S2-15276' exists and 'S2-15286' does not.</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set to 'S2-15286' (one digit off a real WO number).
 2. Inspect the response for a Work Order match.</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr">
         <is>
           <t>1. The real Work Order 'S2-15276' is NOT returned as a fuzzy identifier match.
 2. Identifier fields (VIN, WO number, P-number, part number) require exact match after normalization; fuzzy logic is bypassed for them.</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>requirements.md 7 (What is NOT fuzzy)</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="I80" s="2" t="inlineStr">
         <is>
           <t>GS-API-05</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>GET /api/search enforces role-based access on the server (no forbidden entity results)</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E81" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint as a user whose role does NOT include Parts access.
 2. Parts exist that match the query.</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set to a query that matches parts, and scope set to 'all'.
 2. Inspect the response for a parts group.
 3. Send GET /api/search with scope set to 'parts' as the same restricted user.</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G81" s="2" t="inlineStr">
         <is>
           <t>1. The response contains no parts results for the restricted user (permission filtering is enforced server-side, not just hidden in the UI).
 2. Scoping directly to 'parts' still returns no forbidden parts (empty or a permission-appropriate response).
 3. Entity types the user is allowed to access are still returned.</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>requirements.md 9 (results respect role-based-access checks - enforced server-side)</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
+      <c r="I81" s="2" t="inlineStr">
         <is>
           <t>GS-API-06</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>GET /api/search returns an error response the UI can degrade on</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. You can force an error condition (for example an invalid scope value, or a backend/search-infra failure).</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with an invalid parameter (for example an unknown scope value).
 2. Inspect the HTTP status and error body.
 3. Separately, simulate a backend/search failure and observe the response.</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>1. An invalid request returns an appropriate 4xx status with an error body.
 2. A backend failure returns a 5xx or error payload that the frontend maps to the inline 'Search unavailable, retry' banner (see GS-ERR-01).
 3. The endpoint fails gracefully rather than returning malformed data.</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>requirements.md 8 (offline/network failure handling)</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>GS-API-07</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>GET /api/search groups results in the fixed group order with ranking metadata</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A query matches all six entity types.</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set and scope set to 'all'.
 2. Inspect the order of the groups and the per-item score/rank fields in the response.</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>1. Groups are returned in the order Work Orders, Customers, Assets, Parts, Vendors, Part Sales.
 2. Within each group items are ordered by score descending.
 3. Each item carries the metadata needed to render its row (entity type, primary/secondary fields, status/quantity, score) without extra fetches.</t>
         </is>
       </c>
-      <c r="H81" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.2 (group order); 10 Phase 1 (per-item metadata)</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
+      <c r="I83" s="2" t="inlineStr">
         <is>
           <t>GS-API-08</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>GET /api/search supports cursor pagination for a scoped tab</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A query matches many records of one entity type (more than one page).</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set, scope set to a single entity type, and a limit.
 2. Take the cursor from the response and send GET /api/search again with that cursor.
 3. Compare the two pages of results.</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>1. The first response returns the first page plus a cursor.
 2. Passing the cursor returns the next page of scoped results (no duplicates, no gaps).
 3. Pagination applies to the scoped-tab view.</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>requirements.md 10 Phase 1 (cursor parameter)</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>GS-API-09</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>The context parameter biases GET /api/search ranking to the current page</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>1. You can call the backend search endpoint.
 2. A specific customer owns some assets/work orders; other customers have similar matches.</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>1. Send GET /api/search with q set and no context, and note the ranking of assets/work orders.
 2. Send GET /api/search with q set and context set to {type: customer, id: &lt;that customer&gt;}.
 3. Compare the rankings.</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>1. With the customer context, assets and work orders owned by that customer are boosted in the ranking versus the no-context call.
 2. The context parameter takes an optional {type, id} for page-context bias.</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>requirements.md 6.3 (contextual bias); 10 Phase 1 (context parameter)</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>GS-API-10</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K83" s="2" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>Recent-entities endpoints record and return recent activity</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>1. You can call the recent-entities endpoints with a valid session.</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>1. Send POST /user/recent-entities/touch for a record (for example a work order you opened).
 2. Send GET /user/recent-entities.
 3. Inspect the returned list and its time bucketing.</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t>1. POST /user/recent-entities/touch records the touch (HTTP 2xx).
 2. GET /user/recent-entities returns the recently touched records, retained for 30 days.
 3. The results support bucketing into Today / Yesterday / Past week / Past 30 days at render time.</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>requirements.md 8 (persist recent-entity-views 30 days); 10 Phase 4</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="I86" s="2" t="inlineStr">
         <is>
           <t>GS-API-11</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>API - Global Search Endpoint</t>
         </is>
       </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>Search input is debounced before the backend is queried</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>1. The palette is open.
 2. You can observe outgoing search requests (for example via browser network tools).</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>1. Type a multi-character query quickly without pausing.
 2. Observe how many GET /api/search calls are sent while typing.
 3. Pause typing and observe.</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t>1. The backend is not queried on every keystroke; input is debounced (about 150ms) so a request fires after a short pause.
 2. Grouped results render quickly once the response arrives (target within about 200ms at p95).</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>requirements.md 8 (debounce input at 150ms; render within 200ms p95)</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="I87" s="2" t="inlineStr">
         <is>
           <t>GS-API-12</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>pending push</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>